<commit_message>
Runbook: commands and SQL column, rollback
</commit_message>
<xml_diff>
--- a/Docs/RELEASE-DAY-RUNBOOK.xlsx
+++ b/Docs/RELEASE-DAY-RUNBOOK.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="143">
   <si>
     <t xml:space="preserve">30 Acts of Kindness - release runbook</t>
   </si>
@@ -53,6 +53,9 @@
     <t xml:space="preserve">How you know it worked</t>
   </si>
   <si>
+    <t xml:space="preserve">Command / SQL (copy exactly)</t>
+  </si>
+  <si>
     <t xml:space="preserve">TUESDAY 29 / WEDNESDAY 30 SEPTEMBER - preparation (only you, David and the testers can see any of this)</t>
   </si>
   <si>
@@ -65,18 +68,24 @@
     <t xml:space="preserve">PowerShell</t>
   </si>
   <si>
-    <t xml:space="preserve">Check both logins: npx eas whoami ; npx supabase projects list</t>
+    <t xml:space="preserve">Check both logins.</t>
   </si>
   <si>
     <t xml:space="preserve">Both show you logged in; the list includes mtfyekdxtkdiaqbgaoza.</t>
   </si>
   <si>
-    <t xml:space="preserve">Check the code is clean: git status ; git log -1 --oneline</t>
+    <t xml:space="preserve">npx eas whoami; npx supabase projects list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check the code is clean.</t>
   </si>
   <si>
     <t xml:space="preserve">"working tree clean".</t>
   </si>
   <si>
+    <t xml:space="preserve">git status; git log -1 --oneline</t>
+  </si>
+  <si>
     <t xml:space="preserve">Claude + Chrome</t>
   </si>
   <si>
@@ -101,25 +110,44 @@
     <t xml:space="preserve">WEDNESDAY - reminders deploy (items 27, 28, 51, 52, 61, 66). Approved 29 Sep. Safe at every step: after the deploy the old key still works, so no reminder is missed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Deploy the new reminders code: npx supabase functions deploy send-reminders --project-ref mtfyekdxtkdiaqbgaoza</t>
+    <t xml:space="preserve">PowerShell, in 30-Acts-current</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy the new reminders code (command in the last column).</t>
   </si>
   <si>
     <t xml:space="preserve">"Deployed Function send-reminders".</t>
   </si>
   <si>
+    <t xml:space="preserve">npx supabase functions deploy send-reminders --project-ref mtfyekdxtkdiaqbgaoza</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supabase production - SQL Editor</t>
   </si>
   <si>
-    <t xml:space="preserve">Wait for the next 5-minute tick, then run Claude's check query.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status 200 (old key still works).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create the door secret inside Vault (Claude's query; the database generates it, so it never appears in chat).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The query returns the new secret's id.</t>
+    <t xml:space="preserve">Wait for the next 5-minute tick (:00, :05, :10 ...), then run the check query.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The newest row (latest created time) shows status_code 200.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select id, status_code, created
+from net._http_response
+order by id desc
+limit 5;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create the door secret inside Vault. The database generates it, so it never appears in chat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The query returns an id (a long string of letters and numbers).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select vault.create_secret(
+  encode(extensions.gen_random_bytes(32), 'hex'),
+  'reminders_door_secret',
+  'send-reminders door check (item 52)'
+);</t>
   </si>
   <si>
     <t xml:space="preserve">Supabase production - SQL Editor, then Edge Functions &gt; Secrets</t>
@@ -131,30 +159,53 @@
     <t xml:space="preserve">The secret is listed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Show cron job 7's command; Claude writes the replacement that reads the secret from Vault; run it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command updated.</t>
+    <t xml:space="preserve">select decrypted_secret
+from vault.decrypted_secrets
+where name = 'reminders_door_secret';
+-- Copy the value (never into chat). Then Edge Functions &gt; Secrets &gt; Add new secret:
+-- Name: REMINDERS_DOOR_SECRET   Value: the copied text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point cron job 7 at the new door secret (it also stops sending the admin key).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The query returns one row (no error).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select cron.alter_job(
+  7,
+  command := $cmd$
+  select net.http_post(
+    url     := 'https://mtfyekdxtkdiaqbgaoza.supabase.co/functions/v1/send-reminders',
+    headers := jsonb_build_object(
+      'Content-Type', 'application/json',
+      'apikey',       (select decrypted_secret from vault.decrypted_secrets where name = 'reminders_door_secret')
+    ),
+    body    := '{}'::jsonb,
+    timeout_milliseconds := 30000
+  );
+  $cmd$
+);</t>
   </si>
   <si>
     <t xml:space="preserve">Wait for the next tick and run the check query again.</t>
   </si>
   <si>
-    <t xml:space="preserve">Status 200. (If 401: put the old command back - Claude keeps it.)</t>
+    <t xml:space="preserve">The newest row shows status_code 200. If 401: run the rollback on the second tab.</t>
   </si>
   <si>
     <t xml:space="preserve">WEDNESDAY - 1.0.1 update, then the sign-in hook (items 41, 43, 15, 18, 53, 54, 67, 17c-app, 59). Approved 29 Sep. The update MUST go first: the old sign-in screen does not ask for a code.</t>
   </si>
   <si>
-    <t xml:space="preserve">PowerShell, in 30-Acts-current</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Publish 1.0.1: npx eas update --branch production --environment production -m "1.0.1"</t>
+    <t xml:space="preserve">Publish the 1.0.1 update (command in the last column).</t>
   </si>
   <si>
     <t xml:space="preserve">"Published!" with an update id. Send Claude the id.</t>
   </si>
   <si>
+    <t xml:space="preserve">npx eas update --branch production --environment production -m "1.0.1"</t>
+  </si>
+  <si>
     <t xml:space="preserve">iPhone - production 30 Acts app</t>
   </si>
   <si>
@@ -215,10 +266,10 @@
     <t xml:space="preserve">6:50</t>
   </si>
   <si>
-    <t xml:space="preserve">Run Claude's check query on the overnight reminder ticks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All 200.</t>
+    <t xml:space="preserve">Check the latest reminder ticks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All rows show status_code 200.</t>
   </si>
   <si>
     <t xml:space="preserve">7:00</t>
@@ -392,10 +443,30 @@
     <t xml:space="preserve">What happened</t>
   </si>
   <si>
-    <t xml:space="preserve">A reminder tick returns 401 after the cron change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Put cron job 7's previous command back (Claude keeps it). Reminders resume at the next tick.</t>
+    <t xml:space="preserve">A reminder tick returns 401 after the cron change (step 9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supabase production SQL Editor: run the rollback SQL in the next row. Reminders resume at the next tick. Then tell Claude.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROLLBACK SQL for step 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select cron.alter_job(
+  7,
+  command := $cmd$
+  select net.http_post(
+    url     := 'https://mtfyekdxtkdiaqbgaoza.supabase.co/functions/v1/send-reminders',
+    headers := jsonb_build_object(
+      'Content-Type',  'application/json',
+      'apikey',        (select decrypted_secret from vault.decrypted_secrets where name = 'reminders_secret_key'),
+      'Authorization', concat('Bearer ', (select decrypted_secret from vault.decrypted_secrets where name = 'reminders_secret_key'))
+    ),
+    body    := '{}'::jsonb,
+    timeout_milliseconds := 30000
+  );
+  $cmd$
+);</t>
   </si>
   <si>
     <t xml:space="preserve">Nobody can sign in after the hook is enabled</t>
@@ -429,7 +500,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -521,6 +592,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF1F3A2B"/>
+      <name val="Consolas"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="16"/>
       <color rgb="FF114E33"/>
@@ -528,8 +606,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -539,13 +623,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF114E33"/>
-        <bgColor rgb="FF003366"/>
+        <bgColor rgb="FF1F3A2B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE5F2EA"/>
-        <bgColor rgb="FFCFE7D8"/>
+        <bgColor rgb="FFF4F6F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4F6F3"/>
+        <bgColor rgb="FFE5F2EA"/>
       </patternFill>
     </fill>
   </fills>
@@ -598,7 +688,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -647,7 +737,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -660,6 +754,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -701,7 +799,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFF4F6F3"/>
       <rgbColor rgb="FFE5F2EA"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFEF6F45"/>
@@ -731,14 +829,14 @@
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF114E33"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF114E33"/>
+      <rgbColor rgb="FF1F3A2B"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -924,15 +1022,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -975,106 +1074,119 @@
       <c r="F6" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="G6" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>11</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>10</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>22</v>
+      </c>
+      <c r="G12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8"/>
       <c r="B13" s="9" t="n">
         <v>4</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>23</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="G13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8"/>
@@ -1082,118 +1194,137 @@
         <v>5</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8"/>
       <c r="B17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8"/>
       <c r="B18" s="9" t="n">
         <v>7</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8"/>
       <c r="B19" s="9" t="n">
         <v>8</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="228" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8"/>
       <c r="B20" s="9" t="n">
         <v>9</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>44</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8"/>
       <c r="B21" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>38</v>
+        <v>47</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8"/>
@@ -1201,16 +1332,19 @@
         <v>11</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>42</v>
+        <v>50</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1219,17 +1353,18 @@
         <v>12</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>45</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="G25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8"/>
@@ -1237,17 +1372,18 @@
         <v>13</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>48</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="G26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8"/>
@@ -1255,17 +1391,18 @@
         <v>14</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>51</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="G27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8"/>
@@ -1273,17 +1410,18 @@
         <v>15</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>53</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="G28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8"/>
@@ -1291,63 +1429,69 @@
         <v>16</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>56</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="G29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-    </row>
-    <row r="32" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G31" s="7"/>
+    </row>
+    <row r="32" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8"/>
       <c r="B32" s="9" t="n">
         <v>17</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>70</v>
+      </c>
+      <c r="G32" s="11"/>
+    </row>
+    <row r="33" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="8"/>
       <c r="B33" s="9" t="n">
         <v>18</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>64</v>
+        <v>73</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1356,17 +1500,18 @@
         <v>19</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>68</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="G34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="8"/>
@@ -1374,17 +1519,18 @@
         <v>20</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="G35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="8"/>
@@ -1392,44 +1538,47 @@
         <v>21</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>76</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="G36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="38" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
-    </row>
-    <row r="39" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G38" s="7"/>
+    </row>
+    <row r="39" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="8"/>
       <c r="B39" s="9" t="n">
         <v>22</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>79</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="G39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="8"/>
@@ -1438,46 +1587,49 @@
       </c>
       <c r="C40" s="10"/>
       <c r="D40" s="11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>90</v>
+      </c>
+      <c r="G40" s="11"/>
+    </row>
+    <row r="41" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="8"/>
       <c r="B41" s="9" t="n">
         <v>24</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>92</v>
+      </c>
+      <c r="G41" s="11"/>
+    </row>
+    <row r="42" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="8"/>
       <c r="B42" s="9" t="n">
         <v>25</v>
       </c>
       <c r="C42" s="10"/>
       <c r="D42" s="11" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>85</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="G42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="8"/>
@@ -1486,57 +1638,61 @@
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="11" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>97</v>
+      </c>
+      <c r="G43" s="11"/>
+    </row>
+    <row r="44" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="8"/>
       <c r="B44" s="9" t="n">
         <v>27</v>
       </c>
       <c r="C44" s="10"/>
       <c r="D44" s="11" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>91</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="G44" s="11"/>
     </row>
     <row r="45" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="46" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
-    </row>
-    <row r="47" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G46" s="7"/>
+    </row>
+    <row r="47" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="8"/>
       <c r="B47" s="9" t="n">
         <v>28</v>
       </c>
       <c r="C47" s="10"/>
       <c r="D47" s="11" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>95</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="G47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="8"/>
@@ -1545,14 +1701,15 @@
       </c>
       <c r="C48" s="10"/>
       <c r="D48" s="11" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>97</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="G48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="8"/>
@@ -1561,48 +1718,51 @@
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="11" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>109</v>
+      </c>
+      <c r="G49" s="11"/>
+    </row>
+    <row r="50" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="8"/>
       <c r="B50" s="9" t="n">
         <v>31</v>
       </c>
       <c r="C50" s="10"/>
       <c r="D50" s="11" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+      <c r="G50" s="11"/>
+    </row>
+    <row r="51" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="8"/>
       <c r="B51" s="9" t="n">
         <v>32</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>107</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G51" s="11"/>
     </row>
     <row r="52" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="8"/>
@@ -1610,44 +1770,47 @@
         <v>33</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>111</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="54" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
-    </row>
-    <row r="55" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G54" s="7"/>
+    </row>
+    <row r="55" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="8"/>
       <c r="B55" s="9" t="n">
         <v>34</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="11" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>115</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G55" s="11"/>
     </row>
     <row r="56" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="8"/>
@@ -1655,29 +1818,30 @@
         <v>35</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>119</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="G56" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A54:G54"/>
   </mergeCells>
-  <conditionalFormatting sqref="A10:F56">
+  <conditionalFormatting sqref="A10:G56">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$A10="✓"</formula>
     </cfRule>
@@ -1703,7 +1867,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="45"/>
@@ -1711,56 +1875,64 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>120</v>
+      <c r="A1" s="13" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="13" t="s">
+      <c r="A3" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>125</v>
+      <c r="A4" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="273" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>131</v>
+      <c r="A6" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Runbook: Wednesday steps 5-16 done
</commit_message>
<xml_diff>
--- a/Docs/RELEASE-DAY-RUNBOOK.xlsx
+++ b/Docs/RELEASE-DAY-RUNBOOK.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="143">
   <si>
     <t xml:space="preserve">30 Acts of Kindness - release runbook</t>
   </si>
@@ -1052,7 +1052,7 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="str">
         <f aca="false">"Progress: "&amp;COUNTIF(A10:A56,"✓")&amp;" of "&amp;COUNT(B10:B56)&amp;" steps done"</f>
-        <v>Progress: 3 of 35 steps done</v>
+        <v>Progress: 15 of 35 steps done</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1189,7 +1189,9 @@
       <c r="G15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
+      <c r="A16" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B16" s="9" t="n">
         <v>5</v>
       </c>
@@ -1210,7 +1212,9 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
+      <c r="A17" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B17" s="9" t="n">
         <v>6</v>
       </c>
@@ -1231,7 +1235,9 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
+      <c r="A18" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B18" s="9" t="n">
         <v>7</v>
       </c>
@@ -1252,7 +1258,9 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8"/>
+      <c r="A19" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B19" s="9" t="n">
         <v>8</v>
       </c>
@@ -1273,7 +1281,9 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="228" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8"/>
+      <c r="A20" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B20" s="9" t="n">
         <v>9</v>
       </c>
@@ -1294,7 +1304,9 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8"/>
+      <c r="A21" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B21" s="9" t="n">
         <v>10</v>
       </c>
@@ -1327,7 +1339,9 @@
       <c r="G23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8"/>
+      <c r="A24" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B24" s="9" t="n">
         <v>11</v>
       </c>
@@ -1348,7 +1362,9 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8"/>
+      <c r="A25" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B25" s="9" t="n">
         <v>12</v>
       </c>
@@ -1367,7 +1383,9 @@
       <c r="G25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8"/>
+      <c r="A26" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B26" s="9" t="n">
         <v>13</v>
       </c>
@@ -1386,7 +1404,9 @@
       <c r="G26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8"/>
+      <c r="A27" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B27" s="9" t="n">
         <v>14</v>
       </c>
@@ -1405,7 +1425,9 @@
       <c r="G27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8"/>
+      <c r="A28" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B28" s="9" t="n">
         <v>15</v>
       </c>
@@ -1424,7 +1446,9 @@
       <c r="G28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8"/>
+      <c r="A29" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B29" s="9" t="n">
         <v>16</v>
       </c>

</xml_diff>